<commit_message>
Update data package at: 2025-09-29T17:43:35Z
</commit_message>
<xml_diff>
--- a/data/base_qdd_fiscal_fonte_95.xlsx
+++ b/data/base_qdd_fiscal_fonte_95.xlsx
@@ -488,7 +488,7 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>FUNCAO</t>
+          <t>FUNCAO_COD</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
@@ -5242,13 +5242,13 @@
         <v>1</v>
       </c>
       <c r="V42" t="n">
-        <v>10024937.95</v>
+        <v>10024938</v>
       </c>
       <c r="W42" t="n">
-        <v>10024937.95</v>
+        <v>10024938</v>
       </c>
       <c r="X42" t="n">
-        <v>10024937.95</v>
+        <v>10024938</v>
       </c>
       <c r="Y42" t="n">
         <v>0</v>
@@ -5358,13 +5358,13 @@
         <v>1</v>
       </c>
       <c r="V43" t="n">
-        <v>3392647.75</v>
+        <v>3392647</v>
       </c>
       <c r="W43" t="n">
-        <v>3392647.75</v>
+        <v>3392647</v>
       </c>
       <c r="X43" t="n">
-        <v>3392647.75</v>
+        <v>3392647</v>
       </c>
       <c r="Y43" t="n">
         <v>0</v>
@@ -5472,13 +5472,13 @@
         <v>1</v>
       </c>
       <c r="V44" t="n">
-        <v>10542586.43</v>
+        <v>10542587</v>
       </c>
       <c r="W44" t="n">
-        <v>10542586.43</v>
+        <v>10542587</v>
       </c>
       <c r="X44" t="n">
-        <v>10542586.43</v>
+        <v>10542587</v>
       </c>
       <c r="Y44" t="n">
         <v>0</v>
@@ -5586,13 +5586,13 @@
         <v>1</v>
       </c>
       <c r="V45" t="n">
-        <v>726819.2</v>
+        <v>726819</v>
       </c>
       <c r="W45" t="n">
-        <v>726819.2</v>
+        <v>726819</v>
       </c>
       <c r="X45" t="n">
-        <v>726819.2</v>
+        <v>726819</v>
       </c>
       <c r="Y45" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update data package at: 2025-09-29T17:59:13Z
</commit_message>
<xml_diff>
--- a/data/base_qdd_fiscal_fonte_95.xlsx
+++ b/data/base_qdd_fiscal_fonte_95.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="base_qdd_fiscal" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -49,7 +50,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -412,8 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF68"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -488,7 +488,7 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>FUNCAO_COD</t>
+          <t>FUNCAO</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">

</xml_diff>

<commit_message>
Update data package at: 2025-09-30T11:37:01Z
</commit_message>
<xml_diff>
--- a/data/base_qdd_fiscal_fonte_95.xlsx
+++ b/data/base_qdd_fiscal_fonte_95.xlsx
@@ -413,6 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:AF68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -679,7 +680,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -689,7 +690,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Disponibilização de acesso à água</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Disponibilização de acesso à água</t>
         </is>
       </c>
     </row>
@@ -1365,7 +1366,7 @@
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
@@ -1375,7 +1376,7 @@
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Criação de fundo de disponibilização de crédito para recuperação econômica de pequenas, médias e grandes empresas dos municípios atingidos, além de fundo garantidor para facilitar o acesso a essa linha de crédito</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Criação de fundo de disponibilização de crédito para recuperação econômica de pequenas, médias e grandes empresas dos municípios atingidos, além de fundo garantidor para facilitar o acesso a essa linha de crédito</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1482,7 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
@@ -1491,7 +1492,7 @@
       </c>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Criação de fundo de disponibilização de crédito para recuperação econômica de pequenas, médias e grandes empresas dos municípios atingidos, além de fundo garantidor para facilitar o acesso a essa linha de crédito</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Criação de fundo de disponibilização de crédito para recuperação econômica de pequenas, médias e grandes empresas dos municípios atingidos, além de fundo garantidor para facilitar o acesso a essa linha de crédito</t>
         </is>
       </c>
     </row>
@@ -1597,7 +1598,7 @@
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
@@ -1607,7 +1608,7 @@
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Fomento ao associativismo e ao cooperativismo a partir de assessoria às organizações, podendo incluir aprimoramento da gestão, qualificação de produtos e serviços, apoio na comunicação e marketing, mapeamento de necessidades de infraestrutura e fornecimento de equipamentos e insumos</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Fomento ao associativismo e ao cooperativismo a partir de assessoria às organizações, podendo incluir aprimoramento da gestão, qualificação de produtos e serviços, apoio na comunicação e marketing, mapeamento de necessidades de infraestrutura e fornecimento de equipamentos e insumos</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1714,7 @@
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE11" t="inlineStr">
@@ -1723,7 +1724,7 @@
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Fomento ao associativismo e ao cooperativismo a partir de assessoria às organizações, podendo incluir aprimoramento da gestão, qualificação de produtos e serviços, apoio na comunicação e marketing, mapeamento de necessidades de infraestrutura e fornecimento de equipamentos e insumos</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Fomento ao associativismo e ao cooperativismo a partir de assessoria às organizações, podendo incluir aprimoramento da gestão, qualificação de produtos e serviços, apoio na comunicação e marketing, mapeamento de necessidades de infraestrutura e fornecimento de equipamentos e insumos</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1830,7 @@
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE12" t="inlineStr">
@@ -1839,7 +1840,7 @@
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Fomento ao associativismo e ao cooperativismo a partir de assessoria às organizações, podendo incluir aprimoramento da gestão, qualificação de produtos e serviços, apoio na comunicação e marketing, mapeamento de necessidades de infraestrutura e fornecimento de equipamentos e insumos</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Fomento ao associativismo e ao cooperativismo a partir de assessoria às organizações, podendo incluir aprimoramento da gestão, qualificação de produtos e serviços, apoio na comunicação e marketing, mapeamento de necessidades de infraestrutura e fornecimento de equipamentos e insumos</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1946,7 @@
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE13" t="inlineStr">
@@ -1955,7 +1956,7 @@
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Fomento ao associativismo e ao cooperativismo a partir de assessoria às organizações, podendo incluir aprimoramento da gestão, qualificação de produtos e serviços, apoio na comunicação e marketing, mapeamento de necessidades de infraestrutura e fornecimento de equipamentos e insumos</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Fomento ao associativismo e ao cooperativismo a partir de assessoria às organizações, podendo incluir aprimoramento da gestão, qualificação de produtos e serviços, apoio na comunicação e marketing, mapeamento de necessidades de infraestrutura e fornecimento de equipamentos e insumos</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2062,7 @@
       </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE14" t="inlineStr">
@@ -2071,7 +2072,7 @@
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Fomento ao associativismo e ao cooperativismo a partir de assessoria às organizações, podendo incluir aprimoramento da gestão, qualificação de produtos e serviços, apoio na comunicação e marketing, mapeamento de necessidades de infraestrutura e fornecimento de equipamentos e insumos</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Fomento ao associativismo e ao cooperativismo a partir de assessoria às organizações, podendo incluir aprimoramento da gestão, qualificação de produtos e serviços, apoio na comunicação e marketing, mapeamento de necessidades de infraestrutura e fornecimento de equipamentos e insumos</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2178,7 @@
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE15" t="inlineStr">
@@ -2187,7 +2188,7 @@
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Fomento ao associativismo e ao cooperativismo a partir de assessoria às organizações, podendo incluir aprimoramento da gestão, qualificação de produtos e serviços, apoio na comunicação e marketing, mapeamento de necessidades de infraestrutura e fornecimento de equipamentos e insumos</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Fomento ao associativismo e ao cooperativismo a partir de assessoria às organizações, podendo incluir aprimoramento da gestão, qualificação de produtos e serviços, apoio na comunicação e marketing, mapeamento de necessidades de infraestrutura e fornecimento de equipamentos e insumos</t>
         </is>
       </c>
     </row>
@@ -2293,17 +2294,17 @@
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>A SER CRIADA</t>
+          <t>Fortalecimento dos Serviços de Inspeção Municipais</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 10 - A SER CRIADO - A SER CRIADA</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 10 - INSTRUMENTO A SER CRIADO - Fortalecimento dos Serviços de Inspeção Municipais</t>
         </is>
       </c>
     </row>
@@ -2409,17 +2410,17 @@
       </c>
       <c r="AD17" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>A SER CRIADA</t>
+          <t>Circuitos De Comercialização E Mercados Institucionais</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 10 - A SER CRIADO - A SER CRIADA</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 10 - INSTRUMENTO A SER CRIADO - Circuitos De Comercialização E Mercados Institucionais</t>
         </is>
       </c>
     </row>
@@ -2639,17 +2640,17 @@
       </c>
       <c r="AD19" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>A SER CRIADA</t>
+          <t>Arranjo Produtivo Local Projeto Apicultura</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 10 - A SER CRIADO - A SER CRIADA</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 10 - INSTRUMENTO A SER CRIADO - Arranjo Produtivo Local Projeto Apicultura</t>
         </is>
       </c>
     </row>
@@ -2869,17 +2870,17 @@
       </c>
       <c r="AD21" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>A SER CRIADA</t>
+          <t>Fortalecimento dos Serviços de Inspeção Municipais</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 10 - A SER CRIADO - A SER CRIADA</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 10 - INSTRUMENTO A SER CRIADO - Fortalecimento dos Serviços de Inspeção Municipais</t>
         </is>
       </c>
     </row>
@@ -2985,17 +2986,17 @@
       </c>
       <c r="AD22" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>A SER CRIADA</t>
+          <t>Reestruturação Do Laboratório De Química Agropecuária Do Instituto Mineiro De Agropecuária.</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 10 - A SER CRIADO - A SER CRIADA</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 10 - INSTRUMENTO A SER CRIADO - Reestruturação Do Laboratório De Química Agropecuária Do Instituto Mineiro De Agropecuária.</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3102,7 @@
       </c>
       <c r="AD23" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE23" t="inlineStr">
@@ -3111,7 +3112,7 @@
       </c>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Oferta de serviços de assistência técnica e extensão rural (metodologia ISA/PASEA), visando à produção de alimentos e estímulo à comercialização e adequação socioeconômica e ambiental de propriedades rurais</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Oferta de serviços de assistência técnica e extensão rural (metodologia ISA/PASEA), visando à produção de alimentos e estímulo à comercialização e adequação socioeconômica e ambiental de propriedades rurais</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3218,7 @@
       </c>
       <c r="AD24" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE24" t="inlineStr">
@@ -3227,7 +3228,7 @@
       </c>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Oferta de serviços de assistência técnica e extensão rural (metodologia ISA/PASEA), visando à produção de alimentos e estímulo à comercialização e adequação socioeconômica e ambiental de propriedades rurais</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Oferta de serviços de assistência técnica e extensão rural (metodologia ISA/PASEA), visando à produção de alimentos e estímulo à comercialização e adequação socioeconômica e ambiental de propriedades rurais</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3329,7 @@
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>ANEXO III</t>
         </is>
       </c>
       <c r="AD25" t="n">
@@ -3341,7 +3342,7 @@
       </c>
       <c r="AF25" t="inlineStr">
         <is>
-          <t>Acordo Judicial Vale - III - 9288180 - Implantação do Rodoanel da Região Metropolitana de Belo Horizonte</t>
+          <t>Acordo Judicial Vale - ANEXO III - 9288180 - Implantação do Rodoanel da Região Metropolitana de Belo Horizonte</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3443,7 @@
       </c>
       <c r="AC26" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>ANEXO IV</t>
         </is>
       </c>
       <c r="AD26" t="n">
@@ -3455,7 +3456,7 @@
       </c>
       <c r="AF26" t="inlineStr">
         <is>
-          <t>Acordo Judicial Vale - IV - 9288178 - Prevenção de Enchentes - Construção de Bacias de Contenção no Córrego Ferrugem</t>
+          <t>Acordo Judicial Vale - ANEXO IV - 9288178 - Prevenção de Enchentes - Construção de Bacias de Contenção no Córrego Ferrugem</t>
         </is>
       </c>
     </row>
@@ -3556,7 +3557,7 @@
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>ANEXO IV</t>
         </is>
       </c>
       <c r="AD27" t="n">
@@ -3569,7 +3570,7 @@
       </c>
       <c r="AF27" t="inlineStr">
         <is>
-          <t>Acordo Judicial Vale - IV - 9288179 - Prevenção de Enchentes - Desapropriação para construção de bacias de contenção no Córrego Riacho das Pedras</t>
+          <t>Acordo Judicial Vale - ANEXO IV - 9288179 - Prevenção de Enchentes - Desapropriação para construção de bacias de contenção no Córrego Riacho das Pedras</t>
         </is>
       </c>
     </row>
@@ -4012,7 +4013,7 @@
       </c>
       <c r="AC31" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>ANEXO III</t>
         </is>
       </c>
       <c r="AD31" t="n">
@@ -4025,7 +4026,7 @@
       </c>
       <c r="AF31" t="inlineStr">
         <is>
-          <t>Acordo Judicial Vale - III - 9288132 - Construção de pontes em São Francisco, Manga e São Romão sobre o Rio São Francisco</t>
+          <t>Acordo Judicial Vale - ANEXO III - 9288132 - Construção de pontes em São Francisco, Manga e São Romão sobre o Rio São Francisco</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4127,7 @@
       </c>
       <c r="AC32" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>ANEXO III</t>
         </is>
       </c>
       <c r="AD32" t="n">
@@ -4139,7 +4140,7 @@
       </c>
       <c r="AF32" t="inlineStr">
         <is>
-          <t>Acordo Judicial Vale - III - 9288133 - Recuperação de rodovias pavimentadas em pior estado, conforme avaliação técnica do DER-MG/conclusão de corredor logístico estruturante, conforme critérios técnicos da SEINFRA</t>
+          <t>Acordo Judicial Vale - ANEXO III - 9288133 - Recuperação de rodovias pavimentadas em pior estado, conforme avaliação técnica do DER-MG/conclusão de corredor logístico estruturante, conforme critérios técnicos da SEINFRA</t>
         </is>
       </c>
     </row>
@@ -4582,7 +4583,7 @@
       </c>
       <c r="AC36" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>ANEXO III</t>
         </is>
       </c>
       <c r="AD36" t="n">
@@ -4595,7 +4596,7 @@
       </c>
       <c r="AF36" t="inlineStr">
         <is>
-          <t>Acordo Judicial Vale - III - 9288180 - Implantação do Rodoanel da Região Metropolitana de Belo Horizonte</t>
+          <t>Acordo Judicial Vale - ANEXO III - 9288180 - Implantação do Rodoanel da Região Metropolitana de Belo Horizonte</t>
         </is>
       </c>
     </row>
@@ -4704,12 +4705,12 @@
       </c>
       <c r="AE37" t="inlineStr">
         <is>
-          <t>Políticas e ações de competência e execução direta do ESTADO DE MINAS GERAIS para aplicação em saúde nos municípios  (pendente criação de inciativas)</t>
+          <t>Fortalecimento do Sistema Único de Saúde (SUS)</t>
         </is>
       </c>
       <c r="AF37" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 08 - 9445683 - Políticas e ações de competência e execução direta do ESTADO DE MINAS GERAIS para aplicação em saúde nos municípios  (pendente criação de inciativas)</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 08 - 9445683 - Fortalecimento do Sistema Único de Saúde (SUS)</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4816,7 @@
       </c>
       <c r="AD38" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE38" t="inlineStr">
@@ -4825,7 +4826,7 @@
       </c>
       <c r="AF38" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas ambientais</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas ambientais</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4932,7 @@
       </c>
       <c r="AD39" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE39" t="inlineStr">
@@ -4941,7 +4942,7 @@
       </c>
       <c r="AF39" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Melhoria na capacidade estadual fiscalizatória de barragens nas estruturas localizadas na extensão territorial da Bacia Hidrográfica do Rio Doce: aquisição de equipamentos físicos e tecnológicos, contratação de serviços de consultoria</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Melhoria na capacidade estadual fiscalizatória de barragens nas estruturas localizadas na extensão territorial da Bacia Hidrográfica do Rio Doce: aquisição de equipamentos físicos e tecnológicos, contratação de serviços de consultoria</t>
         </is>
       </c>
     </row>
@@ -5050,12 +5051,12 @@
       </c>
       <c r="AE40" t="inlineStr">
         <is>
-          <t>Consolidação de unidades de conservação estaduais na Bacia Hidrográfica do Rio Doce, a partir do investimento e custeio de suas estruturas e serviços prestados, de acordo com seus objetivos de criação; criação, se necessário, de nova(s) unidade(s) de conservação na Bacia Hidrográfica do Rio Doce de acordo com mapeamento de áreas prioritárias para conservação; realização de atividades de prevenção e combate a incêndios e regularização fundiária das unidades de conservação.</t>
+          <t>Consolidação de unidades de conservação estaduais na Bacia Hidrográfica do Rio Doce, a partir do investimento e custeio de suas estruturas e serviços prestados, de acordo com seus objetivos de criação; criação, se necessário, de nova(s) unidade(s) de conservação na Bacia Hidrográfica do Rio Doce de acordo com mapeamento de áreas prioritárias para conservação; realização de atividades de prevenção e combate a incêndios e regularização fundiária das unidades de conservação</t>
         </is>
       </c>
       <c r="AF40" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9456606 - Consolidação de unidades de conservação estaduais na Bacia Hidrográfica do Rio Doce, a partir do investimento e custeio de suas estruturas e serviços prestados, de acordo com seus objetivos de criação; criação, se necessário, de nova(s) unidade(s) de conservação na Bacia Hidrográfica do Rio Doce de acordo com mapeamento de áreas prioritárias para conservação; realização de atividades de prevenção e combate a incêndios e regularização fundiária das unidades de conservação.</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9456606 - Consolidação de unidades de conservação estaduais na Bacia Hidrográfica do Rio Doce, a partir do investimento e custeio de suas estruturas e serviços prestados, de acordo com seus objetivos de criação; criação, se necessário, de nova(s) unidade(s) de conservação na Bacia Hidrográfica do Rio Doce de acordo com mapeamento de áreas prioritárias para conservação; realização de atividades de prevenção e combate a incêndios e regularização fundiária das unidades de conservação</t>
         </is>
       </c>
     </row>
@@ -5164,12 +5165,12 @@
       </c>
       <c r="AE41" t="inlineStr">
         <is>
-          <t>Consolidação de unidades de conservação estaduais na Bacia Hidrográfica do Rio Doce, a partir do investimento e custeio de suas estruturas e serviços prestados, de acordo com seus objetivos de criação; criação, se necessário, de nova(s) unidade(s) de conservação na Bacia Hidrográfica do Rio Doce de acordo com mapeamento de áreas prioritárias para conservação; realização de atividades de prevenção e combate a incêndios e regularização fundiária das unidades de conservação.</t>
+          <t>Consolidação de unidades de conservação estaduais na Bacia Hidrográfica do Rio Doce, a partir do investimento e custeio de suas estruturas e serviços prestados, de acordo com seus objetivos de criação; criação, se necessário, de nova(s) unidade(s) de conservação na Bacia Hidrográfica do Rio Doce de acordo com mapeamento de áreas prioritárias para conservação; realização de atividades de prevenção e combate a incêndios e regularização fundiária das unidades de conservação</t>
         </is>
       </c>
       <c r="AF41" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9456606 - Consolidação de unidades de conservação estaduais na Bacia Hidrográfica do Rio Doce, a partir do investimento e custeio de suas estruturas e serviços prestados, de acordo com seus objetivos de criação; criação, se necessário, de nova(s) unidade(s) de conservação na Bacia Hidrográfica do Rio Doce de acordo com mapeamento de áreas prioritárias para conservação; realização de atividades de prevenção e combate a incêndios e regularização fundiária das unidades de conservação.</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9456606 - Consolidação de unidades de conservação estaduais na Bacia Hidrográfica do Rio Doce, a partir do investimento e custeio de suas estruturas e serviços prestados, de acordo com seus objetivos de criação; criação, se necessário, de nova(s) unidade(s) de conservação na Bacia Hidrográfica do Rio Doce de acordo com mapeamento de áreas prioritárias para conservação; realização de atividades de prevenção e combate a incêndios e regularização fundiária das unidades de conservação</t>
         </is>
       </c>
     </row>
@@ -5275,7 +5276,7 @@
       </c>
       <c r="AD42" t="inlineStr">
         <is>
-          <t>A CRIAR</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE42" t="inlineStr">
@@ -5285,7 +5286,7 @@
       </c>
       <c r="AF42" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 10 - A CRIAR -  Elaboração e/ou atualização do ordenamento pesqueiro, na forma da Lei n. 11.959, de 29 de junho de 2009. III. Recomposição da biota, dos recursos e dos estoques pesqueiros do ecossistema como um todo na Bacia Hidrográfica do rio Doce, em sua foz e região costeira e marinha.</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 10 - INSTRUMENTO A SER CRIADO -  Elaboração e/ou atualização do ordenamento pesqueiro, na forma da Lei n. 11.959, de 29 de junho de 2009. III. Recomposição da biota, dos recursos e dos estoques pesqueiros do ecossistema como um todo na Bacia Hidrográfica do rio Doce, em sua foz e região costeira e marinha.</t>
         </is>
       </c>
     </row>
@@ -5622,12 +5623,12 @@
       </c>
       <c r="AE45" t="inlineStr">
         <is>
-          <t>Fortalecimento da política pública de gestão do manejo da fauna silvestre, de acordo com mapeamento de necessidades a ser detalhado, a partir de ações como da estruturação e custeio dos serviços prestados porelos Cetras que atendam à bacia hidrográfica do rio Doce; contratação de serviços veterinários especializados; construção de viveiros em áreas de parceiros para a reabilitação e conservação da faun</t>
+          <t>Fortalecimento da política pública de gestão do manejo da fauna silvestre, de acordo com mapeamento de necessidades a ser detalhado, a partir de ações como da estruturação e custeio dos serviços prestados porelos Cetras que atendam à bacia hidrográfica do rio Doce; contratação de serviços veterinários especializados; construção de viveiros em áreas de parceiros para a reabilitação e conservação da faunA</t>
         </is>
       </c>
       <c r="AF45" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9456605 - Fortalecimento da política pública de gestão do manejo da fauna silvestre, de acordo com mapeamento de necessidades a ser detalhado, a partir de ações como da estruturação e custeio dos serviços prestados porelos Cetras que atendam à bacia hidrográfica do rio Doce; contratação de serviços veterinários especializados; construção de viveiros em áreas de parceiros para a reabilitação e conservação da faun</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9456605 - Fortalecimento da política pública de gestão do manejo da fauna silvestre, de acordo com mapeamento de necessidades a ser detalhado, a partir de ações como da estruturação e custeio dos serviços prestados porelos Cetras que atendam à bacia hidrográfica do rio Doce; contratação de serviços veterinários especializados; construção de viveiros em áreas de parceiros para a reabilitação e conservação da faunA</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6190,7 @@
       </c>
       <c r="AD50" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE50" t="inlineStr">
@@ -6199,7 +6200,7 @@
       </c>
       <c r="AF50" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Ampliação, modernização e equipagem da rede meteorológica, rede hidrológica e Sala de Situação para eventos hidrológicos críticos, de forma a aprimorar a capacidade do Sistema Estadual de Meio Ambiente (SISEMA) de acompanhar a recuperação da Bacia Hidrográfica do Rio Doce vis-à-vis riscos decorrentes de eventos climáticos extremos.</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Ampliação, modernização e equipagem da rede meteorológica, rede hidrológica e Sala de Situação para eventos hidrológicos críticos, de forma a aprimorar a capacidade do Sistema Estadual de Meio Ambiente (SISEMA) de acompanhar a recuperação da Bacia Hidrográfica do Rio Doce vis-à-vis riscos decorrentes de eventos climáticos extremos.</t>
         </is>
       </c>
     </row>
@@ -6305,7 +6306,7 @@
       </c>
       <c r="AD51" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE51" t="inlineStr">
@@ -6315,7 +6316,7 @@
       </c>
       <c r="AF51" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Ampliação, modernização e equipagem da rede meteorológica, rede hidrológica e Sala de Situação para eventos hidrológicos críticos, de forma a aprimorar a capacidade do Sistema Estadual de Meio Ambiente (SISEMA) de acompanhar a recuperação da Bacia Hidrográfica do Rio Doce vis-à-vis riscos decorrentes de eventos climáticos extremos.</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Ampliação, modernização e equipagem da rede meteorológica, rede hidrológica e Sala de Situação para eventos hidrológicos críticos, de forma a aprimorar a capacidade do Sistema Estadual de Meio Ambiente (SISEMA) de acompanhar a recuperação da Bacia Hidrográfica do Rio Doce vis-à-vis riscos decorrentes de eventos climáticos extremos.</t>
         </is>
       </c>
     </row>
@@ -6421,7 +6422,7 @@
       </c>
       <c r="AD52" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE52" t="inlineStr">
@@ -6431,7 +6432,7 @@
       </c>
       <c r="AF52" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Ampliação, modernização e equipagem da rede meteorológica, rede hidrológica e Sala de Situação para eventos hidrológicos críticos, de forma a aprimorar a capacidade do Sistema Estadual de Meio Ambiente (SISEMA) de acompanhar a recuperação da Bacia Hidrográfica do Rio Doce vis-à-vis riscos decorrentes de eventos climáticos extremos.</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Ampliação, modernização e equipagem da rede meteorológica, rede hidrológica e Sala de Situação para eventos hidrológicos críticos, de forma a aprimorar a capacidade do Sistema Estadual de Meio Ambiente (SISEMA) de acompanhar a recuperação da Bacia Hidrográfica do Rio Doce vis-à-vis riscos decorrentes de eventos climáticos extremos.</t>
         </is>
       </c>
     </row>
@@ -6537,7 +6538,7 @@
       </c>
       <c r="AD53" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE53" t="inlineStr">
@@ -6547,7 +6548,7 @@
       </c>
       <c r="AF53" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Ampliação, modernização e equipagem da rede meteorológica, rede hidrológica e Sala de Situação para eventos hidrológicos críticos, de forma a aprimorar a capacidade do Sistema Estadual de Meio Ambiente (SISEMA) de acompanhar a recuperação da Bacia Hidrográfica do Rio Doce vis-à-vis riscos decorrentes de eventos climáticos extremos.</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Ampliação, modernização e equipagem da rede meteorológica, rede hidrológica e Sala de Situação para eventos hidrológicos críticos, de forma a aprimorar a capacidade do Sistema Estadual de Meio Ambiente (SISEMA) de acompanhar a recuperação da Bacia Hidrográfica do Rio Doce vis-à-vis riscos decorrentes de eventos climáticos extremos.</t>
         </is>
       </c>
     </row>
@@ -6653,7 +6654,7 @@
       </c>
       <c r="AD54" t="inlineStr">
         <is>
-          <t>A SER CRIADO</t>
+          <t>INSTRUMENTO A SER CRIADO</t>
         </is>
       </c>
       <c r="AE54" t="inlineStr">
@@ -6663,7 +6664,7 @@
       </c>
       <c r="AF54" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - A SER CRIADO - Melhoria na capacidade estadual fiscalizatória de barragens nas estruturas localizadas na extensão territorial da Bacia Hidrográfica do Rio Doce: aquisição de equipamentos físicos e tecnológicos, contratação de serviços de consultoria</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - INSTRUMENTO A SER CRIADO - Melhoria na capacidade estadual fiscalizatória de barragens nas estruturas localizadas na extensão territorial da Bacia Hidrográfica do Rio Doce: aquisição de equipamentos físicos e tecnológicos, contratação de serviços de consultoria</t>
         </is>
       </c>
     </row>
@@ -7000,12 +7001,12 @@
       </c>
       <c r="AE57" t="inlineStr">
         <is>
-          <t>Oferta de cursos de qualificação profissional a partir de estudo de demandas do mercado de trabalho - SEDESE</t>
+          <t>Oferta de cursos de qualificação profissional a partir de estudo de demandas do mercado de trabalho</t>
         </is>
       </c>
       <c r="AF57" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9456621 - Oferta de cursos de qualificação profissional a partir de estudo de demandas do mercado de trabalho - SEDESE</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9456621 - Oferta de cursos de qualificação profissional a partir de estudo de demandas do mercado de trabalho</t>
         </is>
       </c>
     </row>
@@ -7114,12 +7115,12 @@
       </c>
       <c r="AE58" t="inlineStr">
         <is>
-          <t>Oferta de cursos de qualificação profissional a partir de estudo de demandas do mercado de trabalho - SEDESE</t>
+          <t>Oferta de cursos de qualificação profissional a partir de estudo de demandas do mercado de trabalho</t>
         </is>
       </c>
       <c r="AF58" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9456621 - Oferta de cursos de qualificação profissional a partir de estudo de demandas do mercado de trabalho - SEDESE</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9456621 - Oferta de cursos de qualificação profissional a partir de estudo de demandas do mercado de trabalho</t>
         </is>
       </c>
     </row>
@@ -7456,12 +7457,12 @@
       </c>
       <c r="AE61" t="inlineStr">
         <is>
-          <t>Repasse ao Fundo Estadual de Assistência Social (FEAS) do ESTADO DE MINAS GERAIS  (pendente criação de inciativas)</t>
+          <t>Fortalecimento do Sistema Único de Assistência Social (SUAS)</t>
         </is>
       </c>
       <c r="AF61" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 07 - 9445684 - Repasse ao Fundo Estadual de Assistência Social (FEAS) do ESTADO DE MINAS GERAIS  (pendente criação de inciativas)</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 07 - 9445684 - Fortalecimento do Sistema Único de Assistência Social (SUAS)</t>
         </is>
       </c>
     </row>
@@ -7570,12 +7571,12 @@
       </c>
       <c r="AE62" t="inlineStr">
         <is>
-          <t>Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas</t>
+          <t>Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas Lista 3</t>
         </is>
       </c>
       <c r="AF62" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9468055 - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9468055 - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas Lista 3</t>
         </is>
       </c>
     </row>
@@ -7684,12 +7685,12 @@
       </c>
       <c r="AE63" t="inlineStr">
         <is>
-          <t>Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas</t>
+          <t>Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas Lista 3</t>
         </is>
       </c>
       <c r="AF63" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9468055 - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9468055 - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas Lista 3</t>
         </is>
       </c>
     </row>
@@ -7798,12 +7799,12 @@
       </c>
       <c r="AE64" t="inlineStr">
         <is>
-          <t>Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas</t>
+          <t>Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas Lista 3</t>
         </is>
       </c>
       <c r="AF64" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9468055 - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9468055 - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas Lista 3</t>
         </is>
       </c>
     </row>
@@ -7912,12 +7913,12 @@
       </c>
       <c r="AE65" t="inlineStr">
         <is>
-          <t>Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas</t>
+          <t>Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas Lista 3</t>
         </is>
       </c>
       <c r="AF65" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9468055 - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9468055 - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas Lista 3</t>
         </is>
       </c>
     </row>
@@ -8026,12 +8027,12 @@
       </c>
       <c r="AE66" t="inlineStr">
         <is>
-          <t>Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas</t>
+          <t>Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas Lista 3</t>
         </is>
       </c>
       <c r="AF66" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9468055 - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9468055 - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas Lista 3</t>
         </is>
       </c>
     </row>
@@ -8140,12 +8141,12 @@
       </c>
       <c r="AE67" t="inlineStr">
         <is>
-          <t>Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas</t>
+          <t>Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas Lista 3</t>
         </is>
       </c>
       <c r="AF67" t="inlineStr">
         <is>
-          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9468055 - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas</t>
+          <t>Acordo Judicial do Rio Doce - ANEXO 12 - 9468055 - Suporte gerencial, administrativo, tecnológico e de comunicação social à implementação das iniciativas Lista 3</t>
         </is>
       </c>
     </row>

</xml_diff>